<commit_message>
feat: Implement pause functionality and enhance user experience
If applied, this commit will introduce the pause button in the top right corner
of the game screen, allowing users to pause the game at any time. Additionally,
checks have been added in MenuController.java to notify users that exiting
the game during a pause will result in losing progress and not being added to
the leaderboard. An alert box will prompt the user to confirm their decision.

Furthermore, an issue with FoodModel has been resolved. It now properly randomizes
images from 0 to 16, ensuring a wider variety of food images during gameplay.
Obstacles for the snake game will be implemented in upcoming commits, along with
additional functionalities such as new background images triggered by user actions.
</commit_message>
<xml_diff>
--- a/CW2013/local_leaderboard.xlsx
+++ b/CW2013/local_leaderboard.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
   <si>
     <t>Player Name</t>
   </si>
@@ -63,6 +63,18 @@
   </si>
   <si>
     <t>Okd</t>
+  </si>
+  <si>
+    <t>Hello</t>
+  </si>
+  <si>
+    <t>HI</t>
+  </si>
+  <si>
+    <t>John</t>
+  </si>
+  <si>
+    <t>dfasf</t>
   </si>
 </sst>
 </file>
@@ -107,7 +119,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -246,6 +258,38 @@
         <v>3.0</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" t="n">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" t="n">
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" t="n">
+        <v>13.0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" t="n">
+        <v>4.0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Add dynamic background selection and prepare for obstacles
If applied, this commit will introduce a new feature that allows users to
randomly change the game background by pressing the "Change Background" button
in the pause menu. This enhancement aims to make the game more engaging for users.

Additionally, new images for obstacles have been added in preparation for the
upcoming ObstaclesModel implementation. The necessary changes have been made
to Game.FXML, GameController.java, and MenuController.java to support the
background selection functionality.

The ObstaclesModel.java class is planned for implementation
in the upcoming days to fully integrate obstacles into the game.
</commit_message>
<xml_diff>
--- a/CW2013/local_leaderboard.xlsx
+++ b/CW2013/local_leaderboard.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
   <si>
     <t>Player Name</t>
   </si>
@@ -75,6 +75,30 @@
   </si>
   <si>
     <t>dfasf</t>
+  </si>
+  <si>
+    <t>Kolem</t>
+  </si>
+  <si>
+    <t>kjjaksd</t>
+  </si>
+  <si>
+    <t>pkl</t>
+  </si>
+  <si>
+    <t>l</t>
+  </si>
+  <si>
+    <t>ddkadke</t>
+  </si>
+  <si>
+    <t>jj</t>
+  </si>
+  <si>
+    <t>fsdf</t>
+  </si>
+  <si>
+    <t>lol</t>
   </si>
 </sst>
 </file>
@@ -119,7 +143,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -290,6 +314,70 @@
         <v>4.0</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" t="n">
+        <v>21.0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" t="n">
+        <v>8.0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25" t="n">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26" t="n">
+        <v>10.0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27" t="n">
+        <v>19.0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28" t="n">
+        <v>3.0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29" t="n">
+        <v>19.0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
refactor: Generalise ItemsModel and Implement Obstacles Functionality
If applied, this commit will refactor the ItemsModel class to generalise it for different game items. The Obstacle class is removed as it's no longer needed, and instead, the ItemsModel is used for creating obstacles dynamically during the game.

The changes include:
- Refactoring of the ItemsModel class to serve as a common model for various game items, eliminating the need for a separate Obstacle class.
- Implementation of obstacle functionality in the GameController to check for collisions with the snake.
- Deduct bodyPoints from the snake and also from the score, the snake should reduce it's size as it hits the obstacles "lose a life"

Next steps involve creating an ItemsController to manage additional functionalities like slow motion, fast motion, and 2x points power-ups.
</commit_message>
<xml_diff>
--- a/CW2013/local_leaderboard.xlsx
+++ b/CW2013/local_leaderboard.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="48">
   <si>
     <t>Player Name</t>
   </si>
@@ -99,6 +99,63 @@
   </si>
   <si>
     <t>lol</t>
+  </si>
+  <si>
+    <t>i</t>
+  </si>
+  <si>
+    <t>f</t>
+  </si>
+  <si>
+    <t>kl</t>
+  </si>
+  <si>
+    <t>lk</t>
+  </si>
+  <si>
+    <t>g</t>
+  </si>
+  <si>
+    <t>asd</t>
+  </si>
+  <si>
+    <t>asdw</t>
+  </si>
+  <si>
+    <t>asd2</t>
+  </si>
+  <si>
+    <t>ad13</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>f123</t>
+  </si>
+  <si>
+    <t>3414</t>
+  </si>
+  <si>
+    <t>jom</t>
+  </si>
+  <si>
+    <t>e1e13</t>
+  </si>
+  <si>
+    <t>e3</t>
+  </si>
+  <si>
+    <t>de2</t>
+  </si>
+  <si>
+    <t>ee3</t>
+  </si>
+  <si>
+    <t>e2</t>
+  </si>
+  <si>
+    <t>ad</t>
   </si>
 </sst>
 </file>
@@ -143,7 +200,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B52"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -378,6 +435,190 @@
         <v>19.0</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>29</v>
+      </c>
+      <c r="B31" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>30</v>
+      </c>
+      <c r="B32" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>11</v>
+      </c>
+      <c r="B33" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>31</v>
+      </c>
+      <c r="B34" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>11</v>
+      </c>
+      <c r="B35" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>32</v>
+      </c>
+      <c r="B36" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>33</v>
+      </c>
+      <c r="B37" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>34</v>
+      </c>
+      <c r="B38" t="n">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>35</v>
+      </c>
+      <c r="B39" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>36</v>
+      </c>
+      <c r="B40" t="n">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>37</v>
+      </c>
+      <c r="B41" t="n">
+        <v>6.0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>38</v>
+      </c>
+      <c r="B42" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>39</v>
+      </c>
+      <c r="B43" t="n">
+        <v>6.0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>38</v>
+      </c>
+      <c r="B44" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s">
+        <v>40</v>
+      </c>
+      <c r="B45" t="n">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s">
+        <v>41</v>
+      </c>
+      <c r="B46" t="n">
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s">
+        <v>42</v>
+      </c>
+      <c r="B47" t="n">
+        <v>7.0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s">
+        <v>43</v>
+      </c>
+      <c r="B48" t="n">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s">
+        <v>44</v>
+      </c>
+      <c r="B49" t="n">
+        <v>60.0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s">
+        <v>45</v>
+      </c>
+      <c r="B50" t="n">
+        <v>-1.821123914E9</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s">
+        <v>46</v>
+      </c>
+      <c r="B51" t="n">
+        <v>3.09230423E8</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s">
+        <v>47</v>
+      </c>
+      <c r="B52" t="n">
+        <v>8.0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Implement ItemController for enhanced code organization
- Introduce ItemController class to manage game items
- Improve readability in GameController.java by offloading item-related functionalities
- Create methods for handling slow motion, double points, and fast speed items

Additional Details:

- Slow Motion Item:
  - Introduce turtle.png as a slow motion trigger
  - Snake enters slow motion for 5.4 seconds upon collecting the turtle.png item
  - Utilise a timer to control the duration of the slow motion effect
  - Display the turtle.png item after the player reaches 5 score points
  - Reappearance of the turtle.png item is triggered after collecting an additional 10 points

Modified Classes:
- GameController.java
- SnakeModel.java
- ImageUtil.java
</commit_message>
<xml_diff>
--- a/CW2013/local_leaderboard.xlsx
+++ b/CW2013/local_leaderboard.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="57">
   <si>
     <t>Player Name</t>
   </si>
@@ -156,6 +156,33 @@
   </si>
   <si>
     <t>ad</t>
+  </si>
+  <si>
+    <t>e13</t>
+  </si>
+  <si>
+    <t>j</t>
+  </si>
+  <si>
+    <t>kmkl</t>
+  </si>
+  <si>
+    <t>kk</t>
+  </si>
+  <si>
+    <t>dad</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
+    <t>s</t>
+  </si>
+  <si>
+    <t>fd13r1</t>
+  </si>
+  <si>
+    <t>d3</t>
   </si>
 </sst>
 </file>
@@ -200,7 +227,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B52"/>
+  <dimension ref="A1:B70"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -619,6 +646,150 @@
         <v>8.0</v>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="s">
+        <v>48</v>
+      </c>
+      <c r="B53" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s">
+        <v>49</v>
+      </c>
+      <c r="B54" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s">
+        <v>31</v>
+      </c>
+      <c r="B55" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s">
+        <v>50</v>
+      </c>
+      <c r="B56" t="n">
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s">
+        <v>51</v>
+      </c>
+      <c r="B57" t="n">
+        <v>5.0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s">
+        <v>52</v>
+      </c>
+      <c r="B58" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s">
+        <v>53</v>
+      </c>
+      <c r="B59" t="n">
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s">
+        <v>34</v>
+      </c>
+      <c r="B60" t="n">
+        <v>11.0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="s">
+        <v>48</v>
+      </c>
+      <c r="B61" t="n">
+        <v>21.0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s">
+        <v>11</v>
+      </c>
+      <c r="B62" t="n">
+        <v>8.0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s">
+        <v>49</v>
+      </c>
+      <c r="B63" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s">
+        <v>51</v>
+      </c>
+      <c r="B64" t="n">
+        <v>5.0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s">
+        <v>11</v>
+      </c>
+      <c r="B65" t="n">
+        <v>8.0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s">
+        <v>54</v>
+      </c>
+      <c r="B66" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s">
+        <v>51</v>
+      </c>
+      <c r="B67" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s">
+        <v>55</v>
+      </c>
+      <c r="B68" t="n">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s">
+        <v>56</v>
+      </c>
+      <c r="B69" t="n">
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s">
+        <v>11</v>
+      </c>
+      <c r="B70" t="n">
+        <v>1.0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Implement 2x Fast Speed and Progress on Double Points Item in ItemController
- Introduce fast-time.png as a trigger for the 2x fast speed item
- Snake accelerates to double speed upon collecting the fast-time.png item
- Utilise a timer to control the duration of the increased speed effect
- Display the fast-time.png item after the player reaches a specific score threshold
- Define conditions for the reappearance of the fast-time.png item

- Note: Double points implementation is in progress and nearly implemented

Modified Classes:
- GameController.java
- ImageUtil.java
- ItemsModel.java
- ItemsController.java
</commit_message>
<xml_diff>
--- a/CW2013/local_leaderboard.xlsx
+++ b/CW2013/local_leaderboard.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="61">
   <si>
     <t>Player Name</t>
   </si>
@@ -183,6 +183,18 @@
   </si>
   <si>
     <t>d3</t>
+  </si>
+  <si>
+    <t>de</t>
+  </si>
+  <si>
+    <t>d33</t>
+  </si>
+  <si>
+    <t>e</t>
+  </si>
+  <si>
+    <t>fe3</t>
   </si>
 </sst>
 </file>
@@ -227,7 +239,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B70"/>
+  <dimension ref="A1:B74"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -790,6 +802,38 @@
         <v>1.0</v>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" t="s">
+        <v>57</v>
+      </c>
+      <c r="B71" t="n">
+        <v>11.0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="s">
+        <v>58</v>
+      </c>
+      <c r="B72" t="n">
+        <v>23.0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="s">
+        <v>59</v>
+      </c>
+      <c r="B73" t="n">
+        <v>23.0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="s">
+        <v>60</v>
+      </c>
+      <c r="B74" t="n">
+        <v>2.0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Add and Implement Settings Page
If applied, this commit will:
- Introduce SettingsController.java, Settings.fxml, and necessary images (mute.png, volume.png).
- Modify MenuController.java, Menu.fxml to accommodate the new button layout when pausing the game.
- Adjust GameController.java to handle the changes in the game interface.
- Update StageManager.java to support black and white mode and preserve settings throughout gameplay.
- Enhance MusicPlayer.java to include mute and unmute functionality.

This commit brings a fully functional Settings Page to the game, allowing users to adjust settings such as volume, mute, and black and white mode. The code modifications ensure a seamless integration of the new features into the game interface.
</commit_message>
<xml_diff>
--- a/CW2013/local_leaderboard.xlsx
+++ b/CW2013/local_leaderboard.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="84">
   <si>
     <t>Player Name</t>
   </si>
@@ -228,6 +228,42 @@
   </si>
   <si>
     <t>d3d</t>
+  </si>
+  <si>
+    <t>dd</t>
+  </si>
+  <si>
+    <t>r</t>
+  </si>
+  <si>
+    <t>de13</t>
+  </si>
+  <si>
+    <t>3f1</t>
+  </si>
+  <si>
+    <t>3r4</t>
+  </si>
+  <si>
+    <t>d31d3</t>
+  </si>
+  <si>
+    <t>d</t>
+  </si>
+  <si>
+    <t>3e1</t>
+  </si>
+  <si>
+    <t>d13</t>
+  </si>
+  <si>
+    <t>sqaq</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>ded</t>
   </si>
 </sst>
 </file>
@@ -272,7 +308,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B89"/>
+  <dimension ref="A1:B117"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -987,6 +1023,230 @@
         <v>44.0</v>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" t="s">
+        <v>72</v>
+      </c>
+      <c r="B90" t="n">
+        <v>10.0</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="s">
+        <v>46</v>
+      </c>
+      <c r="B91" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="s">
+        <v>11</v>
+      </c>
+      <c r="B92" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="s">
+        <v>73</v>
+      </c>
+      <c r="B93" t="n">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="s">
+        <v>56</v>
+      </c>
+      <c r="B94" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="s">
+        <v>31</v>
+      </c>
+      <c r="B95" t="n">
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="s">
+        <v>11</v>
+      </c>
+      <c r="B96" t="n">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="s">
+        <v>49</v>
+      </c>
+      <c r="B97" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="s">
+        <v>74</v>
+      </c>
+      <c r="B98" t="n">
+        <v>6.0</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="s">
+        <v>56</v>
+      </c>
+      <c r="B99" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="s">
+        <v>43</v>
+      </c>
+      <c r="B100" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="s">
+        <v>75</v>
+      </c>
+      <c r="B101" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="s">
+        <v>56</v>
+      </c>
+      <c r="B102" t="n">
+        <v>12.0</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="s">
+        <v>11</v>
+      </c>
+      <c r="B103" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="s">
+        <v>76</v>
+      </c>
+      <c r="B104" t="n">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="s">
+        <v>77</v>
+      </c>
+      <c r="B105" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="s">
+        <v>57</v>
+      </c>
+      <c r="B106" t="n">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="s">
+        <v>78</v>
+      </c>
+      <c r="B107" t="n">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="s">
+        <v>56</v>
+      </c>
+      <c r="B108" t="n">
+        <v>8.0</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="s">
+        <v>79</v>
+      </c>
+      <c r="B109" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="s">
+        <v>80</v>
+      </c>
+      <c r="B110" t="n">
+        <v>14.0</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="s">
+        <v>43</v>
+      </c>
+      <c r="B111" t="n">
+        <v>3.0</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="s">
+        <v>56</v>
+      </c>
+      <c r="B112" t="n">
+        <v>8.0</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="s">
+        <v>78</v>
+      </c>
+      <c r="B113" t="n">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="s">
+        <v>81</v>
+      </c>
+      <c r="B114" t="n">
+        <v>10.0</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="s">
+        <v>82</v>
+      </c>
+      <c r="B115" t="n">
+        <v>24.0</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="s">
+        <v>56</v>
+      </c>
+      <c r="B116" t="n">
+        <v>11.0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="s">
+        <v>83</v>
+      </c>
+      <c r="B117" t="n">
+        <v>8.0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: Add comprehensive JavaDocs to all classes and methods
If applied, this commit will:
- Introduce new files that are all files generated needed for our JavaDocs
- Fully functional JavaDocs files with many comments and explanation of methods and variables and classes.
</commit_message>
<xml_diff>
--- a/CW2013/local_leaderboard.xlsx
+++ b/CW2013/local_leaderboard.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="88">
   <si>
     <t>Player Name</t>
   </si>
@@ -264,6 +264,18 @@
   </si>
   <si>
     <t>ded</t>
+  </si>
+  <si>
+    <t>31</t>
+  </si>
+  <si>
+    <t>s31</t>
+  </si>
+  <si>
+    <t>f4</t>
+  </si>
+  <si>
+    <t>31e</t>
   </si>
 </sst>
 </file>
@@ -308,7 +320,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B117"/>
+  <dimension ref="A1:B123"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1247,6 +1259,54 @@
         <v>8.0</v>
       </c>
     </row>
+    <row r="118">
+      <c r="A118" t="s">
+        <v>84</v>
+      </c>
+      <c r="B118" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="s">
+        <v>85</v>
+      </c>
+      <c r="B119" t="n">
+        <v>19.0</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="s">
+        <v>43</v>
+      </c>
+      <c r="B120" t="n">
+        <v>18.0</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="s">
+        <v>86</v>
+      </c>
+      <c r="B121" t="n">
+        <v>6.0</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="s">
+        <v>87</v>
+      </c>
+      <c r="B122" t="n">
+        <v>27.0</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="s">
+        <v>56</v>
+      </c>
+      <c r="B123" t="n">
+        <v>7.0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: Prevent music and power-up sound during game pause
If applied, this commit will:
- Modify GameController.java to include checks for game pause status before playing music and power-up sound.
- Update PowerUpModel.java to incorporate pause status check before triggering the sound effect.

This fix ensures that music and power-up sound won't play when the game is paused, addressing the issue of audio playing during pause.
</commit_message>
<xml_diff>
--- a/CW2013/local_leaderboard.xlsx
+++ b/CW2013/local_leaderboard.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="88">
   <si>
     <t>Player Name</t>
   </si>
@@ -320,7 +320,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B123"/>
+  <dimension ref="A1:B124"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1307,6 +1307,14 @@
         <v>7.0</v>
       </c>
     </row>
+    <row r="124">
+      <c r="A124" t="s">
+        <v>56</v>
+      </c>
+      <c r="B124" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Exit button with exit code 0 If applied, this commit will: - Finalise the implementation of the SnakeGame, addressing all known issues. - Ensure smooth and responsive snake movement and control. - Implement exiting the game with exit code 0. - Mark the completion of the Snake Game project.
This commit signifies the successful completion of all project requirements, with the snake operating seamlessly and the game providing a satisfying user experience
</commit_message>
<xml_diff>
--- a/CW2013/local_leaderboard.xlsx
+++ b/CW2013/local_leaderboard.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="107">
   <si>
     <t>Player Name</t>
   </si>
@@ -321,6 +321,18 @@
   </si>
   <si>
     <t>f4f</t>
+  </si>
+  <si>
+    <t>jjr</t>
+  </si>
+  <si>
+    <t>kkk</t>
+  </si>
+  <si>
+    <t>jhkjh</t>
+  </si>
+  <si>
+    <t>kj</t>
   </si>
 </sst>
 </file>
@@ -365,7 +377,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B175"/>
+  <dimension ref="A1:B179"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1768,6 +1780,38 @@
         <v>3.0</v>
       </c>
     </row>
+    <row r="176">
+      <c r="A176" t="s">
+        <v>103</v>
+      </c>
+      <c r="B176" t="n">
+        <v>12.0</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="s">
+        <v>104</v>
+      </c>
+      <c r="B177" t="n">
+        <v>21.0</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="s">
+        <v>105</v>
+      </c>
+      <c r="B178" t="n">
+        <v>5.0</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="s">
+        <v>106</v>
+      </c>
+      <c r="B179" t="n">
+        <v>9.0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>